<commit_message>
Docs: fix line breaks in the internal queries sheet
</commit_message>
<xml_diff>
--- a/docs/NOI-BO-NGUON-VA-TRUY-VAN.xlsx
+++ b/docs/NOI-BO-NGUON-VA-TRUY-VAN.xlsx
@@ -1578,7 +1578,14 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>-- Cũ (SQL Server)\nSELECT CONVERT(char(7), ts_date, 120) AS ym, SUM(time_spent) AS hours, COUNT(DISTINCT ide) AS employees\nFROM Intranet_Warehouse.dbo.Summarized_Timesheet\nGROUP BY CONVERT(char(7), ts_date, 120);\n\n-- Mới (PostgreSQL)\nSELECT to_char(entry_date, 'YYYY-MM') AS ym, SUM(hours) AS hours, COUNT(DISTINCT employee_id) AS employees\nFROM dwh.fact_timesheet\nGROUP BY 1;</t>
+          <t>-- Cũ (SQL Server)
+SELECT CONVERT(char(7), ts_date, 120) AS ym, SUM(time_spent) AS hours, COUNT(DISTINCT ide) AS employees
+FROM Intranet_Warehouse.dbo.Summarized_Timesheet
+GROUP BY CONVERT(char(7), ts_date, 120);
+-- Mới (PostgreSQL)
+SELECT to_char(entry_date, 'YYYY-MM') AS ym, SUM(hours) AS hours, COUNT(DISTINCT employee_id) AS employees
+FROM dwh.fact_timesheet
+GROUP BY 1;</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">

</xml_diff>